<commit_message>
v2 Prompt Round2: force grid cards + role-cards + AI numbering per-person
</commit_message>
<xml_diff>
--- a/語音辨識對照表.xlsx
+++ b/語音辨識對照表.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\錄音檔\meeting-auto\錄音轉會議記錄\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\錄音檔\meeting-auto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214A0320-F77B-41B1-B63B-E101EB3E704D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2685AF-5117-4E44-87E0-7B54A9B93807}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
   <si>
     <t>分類
 （選填）</t>
@@ -151,6 +151,20 @@
   </si>
   <si>
     <t>阿傑</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>進環</t>
+  </si>
+  <si>
+    <t>靖寰</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>電扶</t>
+  </si>
+  <si>
+    <t>電服</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -636,7 +650,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="工作表1"/>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" hidden="1" customWidth="1"/>
@@ -848,7 +862,20 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="6"/>
+      <c r="B16" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>